<commit_message>
feat: complete 2026 labour market analysis update (deck, README, and pipeline
</commit_message>
<xml_diff>
--- a/danish_payroll_data_clean.xlsx
+++ b/danish_payroll_data_clean.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aacc4d0ce77f8a14/Pulpit/Payroll_Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="321" documentId="11_5B832AA9AF77F3225EE56160072C61E795F25B9B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CF2A251-49B5-4657-9882-EF2B410CBC35}"/>
+  <xr:revisionPtr revIDLastSave="388" documentId="11_5B832AA9AF77F3225EE56160072C61E795F25B9B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DE357AA-313E-45F5-9DB9-82347822E8B8}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="14220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="14220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1 - Payroll Trends" sheetId="5" r:id="rId1"/>
-    <sheet name="2 - 2024 Snapshot" sheetId="6" r:id="rId2"/>
-    <sheet name="3 - Growth Rates" sheetId="3" r:id="rId3"/>
+    <sheet name="2 - Payroll Indexed" sheetId="7" r:id="rId2"/>
+    <sheet name="3 - 2024 Snapshot" sheetId="6" r:id="rId3"/>
+    <sheet name="4 - Growth Rates" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="51">
   <si>
     <t>1 Agriculture, forestry and fishing</t>
   </si>
@@ -201,6 +202,12 @@
       </rPr>
       <t xml:space="preserve"> fastest-growing sector at 7.82% average annual payroll growth</t>
     </r>
+  </si>
+  <si>
+    <t>Source: Danmarks Statistik (LONS40 x RAS300) • All industries indexed to 100 in 2013 • Higher value = faster payroll growth</t>
+  </si>
+  <si>
+    <t>Payroll Growth Index by Industry - Denmark 2013-2024, (2013 = 100)</t>
   </si>
 </sst>
 </file>
@@ -350,16 +357,16 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -834,7 +841,7 @@
       <c r="A6" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="C6" s="7">
@@ -878,7 +885,7 @@
       <c r="A7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C7" s="7">
@@ -922,7 +929,7 @@
       <c r="A8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="7" t="s">
         <v>39</v>
       </c>
       <c r="C8" s="7">
@@ -966,7 +973,7 @@
       <c r="A9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="7" t="s">
         <v>40</v>
       </c>
       <c r="C9" s="7">
@@ -1010,7 +1017,7 @@
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="7" t="s">
         <v>41</v>
       </c>
       <c r="C10" s="7">
@@ -1054,7 +1061,7 @@
       <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="7" t="s">
         <v>42</v>
       </c>
       <c r="C11" s="7">
@@ -1098,7 +1105,7 @@
       <c r="A12" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="7" t="s">
         <v>43</v>
       </c>
       <c r="C12" s="7">
@@ -1142,7 +1149,7 @@
       <c r="A13" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="7" t="s">
         <v>44</v>
       </c>
       <c r="C13" s="7">
@@ -1183,7 +1190,7 @@
       </c>
     </row>
     <row r="15" spans="1:14" ht="16.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="18" t="s">
         <v>48</v>
       </c>
       <c r="B15" s="8"/>
@@ -1194,6 +1201,612 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E96EE67-8E8F-44F1-A6C7-E917D16094B4}">
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.81640625" customWidth="1"/>
+    <col min="3" max="3" width="10.453125" customWidth="1"/>
+    <col min="4" max="4" width="10.26953125" customWidth="1"/>
+    <col min="5" max="5" width="9.6328125" customWidth="1"/>
+    <col min="6" max="6" width="10.54296875" customWidth="1"/>
+    <col min="7" max="7" width="10.08984375" customWidth="1"/>
+    <col min="8" max="8" width="9.08984375" customWidth="1"/>
+    <col min="9" max="9" width="9.54296875" customWidth="1"/>
+    <col min="10" max="10" width="9.08984375" customWidth="1"/>
+    <col min="11" max="11" width="9.7265625" customWidth="1"/>
+    <col min="12" max="12" width="8.7265625" customWidth="1"/>
+    <col min="13" max="13" width="8.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="26.5" x14ac:dyDescent="0.9">
+      <c r="A1" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="17" x14ac:dyDescent="0.6">
+      <c r="A2" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="18.5" x14ac:dyDescent="0.65">
+      <c r="A3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="7">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C4" s="19">
+        <f>'1 - Payroll Trends'!D4/'1 - Payroll Trends'!$C$4*100</f>
+        <v>100.0326477309827</v>
+      </c>
+      <c r="D4" s="19">
+        <f>'1 - Payroll Trends'!E4/'1 - Payroll Trends'!$C$4*100</f>
+        <v>100.94678419849821</v>
+      </c>
+      <c r="E4" s="19">
+        <f>'1 - Payroll Trends'!F4/'1 - Payroll Trends'!$C$4*100</f>
+        <v>103.72184133202742</v>
+      </c>
+      <c r="F4" s="19">
+        <f>'1 - Payroll Trends'!G4/'1 - Payroll Trends'!$C$4*100</f>
+        <v>103.52595494613126</v>
+      </c>
+      <c r="G4" s="19">
+        <f>'1 - Payroll Trends'!H4/'1 - Payroll Trends'!$C4*100</f>
+        <v>111.10022853411689</v>
+      </c>
+      <c r="H4" s="19">
+        <f>'1 - Payroll Trends'!I4/'1 - Payroll Trends'!$C4*100</f>
+        <v>114.39764936336925</v>
+      </c>
+      <c r="I4" s="19">
+        <f>'1 - Payroll Trends'!J4/'1 - Payroll Trends'!$C4*100</f>
+        <v>113.48351289585375</v>
+      </c>
+      <c r="J4" s="19">
+        <f>'1 - Payroll Trends'!K4/'1 - Payroll Trends'!$C4*100</f>
+        <v>113.15703558602677</v>
+      </c>
+      <c r="K4" s="19">
+        <f>'1 - Payroll Trends'!L4/'1 - Payroll Trends'!$C4*100</f>
+        <v>121.18837740777015</v>
+      </c>
+      <c r="L4" s="19">
+        <f>'1 - Payroll Trends'!M4/'1 - Payroll Trends'!$C4*100</f>
+        <v>121.8086842964414</v>
+      </c>
+      <c r="M4" s="19">
+        <f>'1 - Payroll Trends'!N4/'1 - Payroll Trends'!$C4*100</f>
+        <v>124.61638916095332</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="10">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C5" s="20">
+        <f>'1 - Payroll Trends'!D5/'1 - Payroll Trends'!C5*100</f>
+        <v>103.42406206112487</v>
+      </c>
+      <c r="D5" s="20">
+        <f>'1 - Payroll Trends'!E5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>105.55072560690164</v>
+      </c>
+      <c r="E5" s="20">
+        <f>'1 - Payroll Trends'!F5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>110.27887380458772</v>
+      </c>
+      <c r="F5" s="20">
+        <f>'1 - Payroll Trends'!G5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>114.20450745669766</v>
+      </c>
+      <c r="G5" s="20">
+        <f>'1 - Payroll Trends'!H5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>119.51447869992644</v>
+      </c>
+      <c r="H5" s="20">
+        <f>'1 - Payroll Trends'!I5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>124.12893733698924</v>
+      </c>
+      <c r="I5" s="20">
+        <f>'1 - Payroll Trends'!J5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>123.92162107938208</v>
+      </c>
+      <c r="J5" s="20">
+        <f>'1 - Payroll Trends'!K5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>132.54865244432554</v>
+      </c>
+      <c r="K5" s="20">
+        <f>'1 - Payroll Trends'!L5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>141.63044205176217</v>
+      </c>
+      <c r="L5" s="20">
+        <f>'1 - Payroll Trends'!M5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>153.0328362201565</v>
+      </c>
+      <c r="M5" s="20">
+        <f>'1 - Payroll Trends'!N5/'1 - Payroll Trends'!$C$5*100</f>
+        <v>165.00367819166721</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="7">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C6" s="19">
+        <f>'1 - Payroll Trends'!D6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>104.72343070229957</v>
+      </c>
+      <c r="D6" s="19">
+        <f>'1 - Payroll Trends'!E6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>111.0783095090118</v>
+      </c>
+      <c r="E6" s="19">
+        <f>'1 - Payroll Trends'!F6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>115.72405220633935</v>
+      </c>
+      <c r="F6" s="19">
+        <f>'1 - Payroll Trends'!G6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>123.38408949658172</v>
+      </c>
+      <c r="G6" s="19">
+        <f>'1 - Payroll Trends'!H6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>131.57240522063393</v>
+      </c>
+      <c r="H6" s="19">
+        <f>'1 - Payroll Trends'!I6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>133.46799254195153</v>
+      </c>
+      <c r="I6" s="19">
+        <f>'1 - Payroll Trends'!J6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>139.4810441267868</v>
+      </c>
+      <c r="J6" s="19">
+        <f>'1 - Payroll Trends'!K6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>151.18085767557488</v>
+      </c>
+      <c r="K6" s="19">
+        <f>'1 - Payroll Trends'!L6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>156.91423244251087</v>
+      </c>
+      <c r="L6" s="19">
+        <f>'1 - Payroll Trends'!M6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>162.60099440646366</v>
+      </c>
+      <c r="M6" s="19">
+        <f>'1 - Payroll Trends'!N6/'1 - Payroll Trends'!$C$6*100</f>
+        <v>172.59167184586698</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="7">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C7" s="19">
+        <f>'1 - Payroll Trends'!D7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>102.11628746840016</v>
+      </c>
+      <c r="D7" s="19">
+        <f>'1 - Payroll Trends'!E7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>105.53268327916217</v>
+      </c>
+      <c r="E7" s="19">
+        <f>'1 - Payroll Trends'!F7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>107.11809317443122</v>
+      </c>
+      <c r="F7" s="19">
+        <f>'1 - Payroll Trends'!G7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>110.84868183459733</v>
+      </c>
+      <c r="G7" s="19">
+        <f>'1 - Payroll Trends'!H7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>116.07800650054172</v>
+      </c>
+      <c r="H7" s="19">
+        <f>'1 - Payroll Trends'!I7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>119.60635608522934</v>
+      </c>
+      <c r="I7" s="19">
+        <f>'1 - Payroll Trends'!J7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>117.62369086312749</v>
+      </c>
+      <c r="J7" s="19">
+        <f>'1 - Payroll Trends'!K7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>126.17551462621886</v>
+      </c>
+      <c r="K7" s="19">
+        <f>'1 - Payroll Trends'!L7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>131.78042614662334</v>
+      </c>
+      <c r="L7" s="19">
+        <f>'1 - Payroll Trends'!M7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>136.92307692307693</v>
+      </c>
+      <c r="M7" s="19">
+        <f>'1 - Payroll Trends'!N7/'1 - Payroll Trends'!$C$7*100</f>
+        <v>143.62224629830266</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="7">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C8" s="19">
+        <f>'1 - Payroll Trends'!D8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>102.20338983050847</v>
+      </c>
+      <c r="D8" s="19">
+        <f>'1 - Payroll Trends'!E8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>108.61016949152543</v>
+      </c>
+      <c r="E8" s="19">
+        <f>'1 - Payroll Trends'!F8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>111.28813559322033</v>
+      </c>
+      <c r="F8" s="19">
+        <f>'1 - Payroll Trends'!G8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>115.06779661016948</v>
+      </c>
+      <c r="G8" s="19">
+        <f>'1 - Payroll Trends'!H8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>121.16949152542371</v>
+      </c>
+      <c r="H8" s="19">
+        <f>'1 - Payroll Trends'!I8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>127.42372881355932</v>
+      </c>
+      <c r="I8" s="19">
+        <f>'1 - Payroll Trends'!J8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>129.40677966101694</v>
+      </c>
+      <c r="J8" s="19">
+        <f>'1 - Payroll Trends'!K8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>139.42372881355934</v>
+      </c>
+      <c r="K8" s="19">
+        <f>'1 - Payroll Trends'!L8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>148.20338983050846</v>
+      </c>
+      <c r="L8" s="19">
+        <f>'1 - Payroll Trends'!M8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>154.66101694915255</v>
+      </c>
+      <c r="M8" s="19">
+        <f>'1 - Payroll Trends'!N8/'1 - Payroll Trends'!$C$8*100</f>
+        <v>159.88135593220338</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="7">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C9" s="19">
+        <f>'1 - Payroll Trends'!D9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>100.33497536945812</v>
+      </c>
+      <c r="D9" s="19">
+        <f>'1 - Payroll Trends'!E9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>102.64039408866996</v>
+      </c>
+      <c r="E9" s="19">
+        <f>'1 - Payroll Trends'!F9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>105.39901477832512</v>
+      </c>
+      <c r="F9" s="19">
+        <f>'1 - Payroll Trends'!G9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>111.03448275862068</v>
+      </c>
+      <c r="G9" s="19">
+        <f>'1 - Payroll Trends'!H9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>117.97044334975368</v>
+      </c>
+      <c r="H9" s="19">
+        <f>'1 - Payroll Trends'!I9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>122.32512315270935</v>
+      </c>
+      <c r="I9" s="19">
+        <f>'1 - Payroll Trends'!J9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>123.84236453201972</v>
+      </c>
+      <c r="J9" s="19">
+        <f>'1 - Payroll Trends'!K9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>127.50738916256157</v>
+      </c>
+      <c r="K9" s="19">
+        <f>'1 - Payroll Trends'!L9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>134.16748768472908</v>
+      </c>
+      <c r="L9" s="19">
+        <f>'1 - Payroll Trends'!M9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>143.70443349753697</v>
+      </c>
+      <c r="M9" s="19">
+        <f>'1 - Payroll Trends'!N9/'1 - Payroll Trends'!$C$9*100</f>
+        <v>153.65517241379311</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="7">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C10" s="19">
+        <f>'1 - Payroll Trends'!D10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>103.4</v>
+      </c>
+      <c r="D10" s="19">
+        <f>'1 - Payroll Trends'!E10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>106.60000000000001</v>
+      </c>
+      <c r="E10" s="19">
+        <f>'1 - Payroll Trends'!F10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>109.60000000000001</v>
+      </c>
+      <c r="F10" s="19">
+        <f>'1 - Payroll Trends'!G10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>114.04999999999998</v>
+      </c>
+      <c r="G10" s="19">
+        <f>'1 - Payroll Trends'!H10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>119.9</v>
+      </c>
+      <c r="H10" s="19">
+        <f>'1 - Payroll Trends'!I10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>125.05000000000001</v>
+      </c>
+      <c r="I10" s="19">
+        <f>'1 - Payroll Trends'!J10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>127.55000000000001</v>
+      </c>
+      <c r="J10" s="19">
+        <f>'1 - Payroll Trends'!K10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>134.5</v>
+      </c>
+      <c r="K10" s="19">
+        <f>'1 - Payroll Trends'!L10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>137.75</v>
+      </c>
+      <c r="L10" s="19">
+        <f>'1 - Payroll Trends'!M10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>142.44999999999999</v>
+      </c>
+      <c r="M10" s="19">
+        <f>'1 - Payroll Trends'!N10/'1 - Payroll Trends'!$C$10*100</f>
+        <v>151.95000000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A11" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="7">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C11" s="19">
+        <f>'1 - Payroll Trends'!D11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>104.09327172971412</v>
+      </c>
+      <c r="D11" s="19">
+        <f>'1 - Payroll Trends'!E11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>108.83626913081142</v>
+      </c>
+      <c r="E11" s="19">
+        <f>'1 - Payroll Trends'!F11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>113.31215708922899</v>
+      </c>
+      <c r="F11" s="19">
+        <f>'1 - Payroll Trends'!G11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>118.6254692463182</v>
+      </c>
+      <c r="G11" s="19">
+        <f>'1 - Payroll Trends'!H11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>125.721917412648</v>
+      </c>
+      <c r="H11" s="19">
+        <f>'1 - Payroll Trends'!I11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>127.28847819809413</v>
+      </c>
+      <c r="I11" s="19">
+        <f>'1 - Payroll Trends'!J11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>128.1980941380306</v>
+      </c>
+      <c r="J11" s="19">
+        <f>'1 - Payroll Trends'!K11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>138.47097892001153</v>
+      </c>
+      <c r="K11" s="19">
+        <f>'1 - Payroll Trends'!L11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>150.2526710944268</v>
+      </c>
+      <c r="L11" s="19">
+        <f>'1 - Payroll Trends'!M11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>160.75656944845508</v>
+      </c>
+      <c r="M11" s="19">
+        <f>'1 - Payroll Trends'!N11/'1 - Payroll Trends'!$C$11*100</f>
+        <v>170.49523534507651</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A12" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="7">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C12" s="19">
+        <f>'1 - Payroll Trends'!D12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>101.49062267491085</v>
+      </c>
+      <c r="D12" s="19">
+        <f>'1 - Payroll Trends'!E12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>103.68422402955591</v>
+      </c>
+      <c r="E12" s="19">
+        <f>'1 - Payroll Trends'!F12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>105.40318649459938</v>
+      </c>
+      <c r="F12" s="19">
+        <f>'1 - Payroll Trends'!G12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>108.39469430689894</v>
+      </c>
+      <c r="G12" s="19">
+        <f>'1 - Payroll Trends'!H12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>112.12766503322473</v>
+      </c>
+      <c r="H12" s="19">
+        <f>'1 - Payroll Trends'!I12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>115.12686969238271</v>
+      </c>
+      <c r="I12" s="19">
+        <f>'1 - Payroll Trends'!J12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>120.66603381481387</v>
+      </c>
+      <c r="J12" s="19">
+        <f>'1 - Payroll Trends'!K12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>125.43038202016574</v>
+      </c>
+      <c r="K12" s="19">
+        <f>'1 - Payroll Trends'!L12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>131.74436205967623</v>
+      </c>
+      <c r="L12" s="19">
+        <f>'1 - Payroll Trends'!M12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>135.718500654232</v>
+      </c>
+      <c r="M12" s="19">
+        <f>'1 - Payroll Trends'!N12/'1 - Payroll Trends'!$C$12*100</f>
+        <v>143.15878595068887</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A13" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="7">
+        <f>100</f>
+        <v>100</v>
+      </c>
+      <c r="C13" s="19">
+        <f>'1 - Payroll Trends'!D13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>100.05172413793105</v>
+      </c>
+      <c r="D13" s="19">
+        <f>'1 - Payroll Trends'!E13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>100.48275862068965</v>
+      </c>
+      <c r="E13" s="19">
+        <f>'1 - Payroll Trends'!F13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>104</v>
+      </c>
+      <c r="F13" s="19">
+        <f>'1 - Payroll Trends'!G13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>108.5</v>
+      </c>
+      <c r="G13" s="19">
+        <f>'1 - Payroll Trends'!H13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>113.98275862068965</v>
+      </c>
+      <c r="H13" s="19">
+        <f>'1 - Payroll Trends'!I13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>117.93103448275863</v>
+      </c>
+      <c r="I13" s="19">
+        <f>'1 - Payroll Trends'!J13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>116.79310344827584</v>
+      </c>
+      <c r="J13" s="19">
+        <f>'1 - Payroll Trends'!K13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>122.00000000000001</v>
+      </c>
+      <c r="K13" s="19">
+        <f>'1 - Payroll Trends'!L13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>128.74137931034483</v>
+      </c>
+      <c r="L13" s="19">
+        <f>'1 - Payroll Trends'!M13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>135.9655172413793</v>
+      </c>
+      <c r="M13" s="19">
+        <f>'1 - Payroll Trends'!N13/'1 - Payroll Trends'!$C$13*100</f>
+        <v>144.48275862068965</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD81825A-1D2C-4E32-A8F7-563D9D802D03}">
   <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1242,7 +1855,7 @@
       <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="7" t="s">
         <v>40</v>
       </c>
       <c r="C4" s="7">
@@ -1262,7 +1875,7 @@
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>39</v>
       </c>
       <c r="C5" s="7">
@@ -1302,7 +1915,7 @@
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="7" t="s">
         <v>42</v>
       </c>
       <c r="C7" s="7">
@@ -1322,7 +1935,7 @@
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="7" t="s">
         <v>41</v>
       </c>
       <c r="C8" s="7">
@@ -1342,7 +1955,7 @@
       <c r="A9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="7" t="s">
         <v>43</v>
       </c>
       <c r="C9" s="7">
@@ -1362,7 +1975,7 @@
       <c r="A10" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="7" t="s">
         <v>36</v>
       </c>
       <c r="C10" s="7">
@@ -1382,7 +1995,7 @@
       <c r="A11" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="7" t="s">
         <v>37</v>
       </c>
       <c r="C11" s="7">
@@ -1402,7 +2015,7 @@
       <c r="A12" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="7" t="s">
         <v>44</v>
       </c>
       <c r="C12" s="7">
@@ -1422,7 +2035,7 @@
       <c r="A13" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="7" t="s">
         <v>45</v>
       </c>
       <c r="C13" s="7">
@@ -1446,7 +2059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>